<commit_message>
Update Implementation Guide JSON file path b414c27dc396882adabf54f9a444461ecbaa3d41
</commit_message>
<xml_diff>
--- a/MAJSushiConfig/ig/FRAdvanceDirectiveLMCDAFHIR.xlsx
+++ b/MAJSushiConfig/ig/FRAdvanceDirectiveLMCDAFHIR.xlsx
@@ -27,7 +27,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/metier/document-core/ConceptMap/FRAdvanceDirectiveLMCDAFHIR</t>
+    <t>https://interop.esante.gouv.fr/ig/document-core/ConceptMap/FRAdvanceDirectiveLMCDAFHIR</t>
   </si>
   <si>
     <t>Version</t>
@@ -63,7 +63,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-07T10:25:17+00:00</t>
+    <t>2026-09-07T11:26:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -108,7 +108,7 @@
     <t>Target</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/document-core/StructureDefinition/FRLMAdvanceDirective</t>
+    <t>https://interop.esante.gouv.fr/ig/document-core/StructureDefinition/FRLMAdvanceDirective|0.1.0</t>
   </si>
   <si>
     <t/>
@@ -201,7 +201,7 @@
     <t>Consent.source[x]</t>
   </si>
   <si>
-    <t>https://interop.esante.gouv.fr/ig/document-core/StructureDefinition/FRLMAttachment</t>
+    <t>https://interop.esante.gouv.fr/ig/document-core/StructureDefinition/FRLMAttachment|0.1.0</t>
   </si>
   <si>
     <t>FRLMAttachment.url</t>

</xml_diff>